<commit_message>
Fixed Gamma, GAB, Alpha, and Fluorescence fully. Get to work on ICPMS, FIMS, LSC.
</commit_message>
<xml_diff>
--- a/Alike Columns.xlsx
+++ b/Alike Columns.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28324"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28526"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\kgmon\OneDrive\Desktop\LIMS\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\kaleb\Desktop\LIMS\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{9447DD7B-48F2-4420-AC44-A3C3850B9181}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{11B78F9B-F6AB-47E9-8D63-0D7AF3E01E7E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{360149B4-E1F2-4E19-BB44-4713DD98EAB8}"/>
+    <workbookView xWindow="-315" yWindow="-16320" windowWidth="29040" windowHeight="16440" xr2:uid="{360149B4-E1F2-4E19-BB44-4713DD98EAB8}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -102,7 +102,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="2" x14ac:knownFonts="1">
+  <fonts count="3" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -117,8 +117,15 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <sz val="11"/>
+      <color theme="0"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
-  <fills count="3">
+  <fills count="4">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -128,6 +135,12 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="FFC6EFCE"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="1" tint="0.14999847407452621"/>
+        <bgColor indexed="64"/>
       </patternFill>
     </fill>
   </fills>
@@ -144,9 +157,11 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="1"/>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="0" xfId="1" applyFont="1" applyFill="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Good" xfId="1" builtinId="26"/>
@@ -485,26 +500,29 @@
   <dimension ref="B1:G17"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="2" max="2" width="17" bestFit="1" customWidth="1"/>
-    <col min="4" max="7" width="17" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="9.140625" style="2"/>
+    <col min="2" max="2" width="17" style="2" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="9.140625" style="2"/>
+    <col min="4" max="7" width="17" style="2" bestFit="1" customWidth="1"/>
+    <col min="8" max="16384" width="9.140625" style="2"/>
   </cols>
   <sheetData>
     <row r="1" spans="2:7" x14ac:dyDescent="0.25">
-      <c r="D1" t="s">
+      <c r="D1" s="2" t="s">
         <v>16</v>
       </c>
-      <c r="E1" t="s">
+      <c r="E1" s="2" t="s">
         <v>17</v>
       </c>
-      <c r="F1" t="s">
+      <c r="F1" s="2" t="s">
         <v>18</v>
       </c>
-      <c r="G1" t="s">
+      <c r="G1" s="2" t="s">
         <v>19</v>
       </c>
     </row>
     <row r="2" spans="2:7" x14ac:dyDescent="0.25">
-      <c r="B2" t="s">
+      <c r="B2" s="2" t="s">
         <v>0</v>
       </c>
       <c r="D2" s="1" t="s">
@@ -513,7 +531,7 @@
       <c r="E2" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="F2" t="s">
+      <c r="F2" s="1" t="s">
         <v>0</v>
       </c>
       <c r="G2" s="1" t="s">
@@ -521,7 +539,7 @@
       </c>
     </row>
     <row r="3" spans="2:7" x14ac:dyDescent="0.25">
-      <c r="B3" t="s">
+      <c r="B3" s="2" t="s">
         <v>1</v>
       </c>
       <c r="D3" s="1" t="s">
@@ -530,7 +548,7 @@
       <c r="E3" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="F3" t="s">
+      <c r="F3" s="1" t="s">
         <v>1</v>
       </c>
       <c r="G3" s="1" t="s">
@@ -538,7 +556,7 @@
       </c>
     </row>
     <row r="4" spans="2:7" x14ac:dyDescent="0.25">
-      <c r="B4" t="s">
+      <c r="B4" s="2" t="s">
         <v>2</v>
       </c>
       <c r="D4" s="1" t="s">
@@ -547,7 +565,7 @@
       <c r="E4" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="F4" t="s">
+      <c r="F4" s="1" t="s">
         <v>2</v>
       </c>
       <c r="G4" s="1" t="s">
@@ -555,7 +573,7 @@
       </c>
     </row>
     <row r="5" spans="2:7" x14ac:dyDescent="0.25">
-      <c r="B5" t="s">
+      <c r="B5" s="2" t="s">
         <v>3</v>
       </c>
       <c r="D5" s="1" t="s">
@@ -564,7 +582,7 @@
       <c r="E5" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="F5" t="s">
+      <c r="F5" s="1" t="s">
         <v>3</v>
       </c>
       <c r="G5" s="1" t="s">
@@ -572,7 +590,7 @@
       </c>
     </row>
     <row r="6" spans="2:7" x14ac:dyDescent="0.25">
-      <c r="B6" t="s">
+      <c r="B6" s="2" t="s">
         <v>4</v>
       </c>
       <c r="D6" s="1" t="s">
@@ -581,7 +599,7 @@
       <c r="E6" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="F6" t="s">
+      <c r="F6" s="1" t="s">
         <v>4</v>
       </c>
       <c r="G6" s="1" t="s">
@@ -589,7 +607,7 @@
       </c>
     </row>
     <row r="7" spans="2:7" x14ac:dyDescent="0.25">
-      <c r="B7" t="s">
+      <c r="B7" s="2" t="s">
         <v>5</v>
       </c>
       <c r="D7" s="1" t="s">
@@ -598,7 +616,7 @@
       <c r="E7" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="F7" t="s">
+      <c r="F7" s="1" t="s">
         <v>5</v>
       </c>
       <c r="G7" s="1" t="s">
@@ -606,7 +624,7 @@
       </c>
     </row>
     <row r="8" spans="2:7" x14ac:dyDescent="0.25">
-      <c r="B8" t="s">
+      <c r="B8" s="2" t="s">
         <v>10</v>
       </c>
       <c r="D8" s="1" t="s">
@@ -615,7 +633,7 @@
       <c r="E8" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="F8" t="s">
+      <c r="F8" s="1" t="s">
         <v>10</v>
       </c>
       <c r="G8" s="1" t="s">
@@ -623,7 +641,7 @@
       </c>
     </row>
     <row r="9" spans="2:7" x14ac:dyDescent="0.25">
-      <c r="B9" t="s">
+      <c r="B9" s="2" t="s">
         <v>6</v>
       </c>
       <c r="D9" s="1" t="s">
@@ -632,7 +650,7 @@
       <c r="E9" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="F9" t="s">
+      <c r="F9" s="1" t="s">
         <v>6</v>
       </c>
       <c r="G9" s="1" t="s">
@@ -640,7 +658,7 @@
       </c>
     </row>
     <row r="10" spans="2:7" x14ac:dyDescent="0.25">
-      <c r="B10" t="s">
+      <c r="B10" s="2" t="s">
         <v>7</v>
       </c>
       <c r="D10" s="1" t="s">
@@ -649,7 +667,7 @@
       <c r="E10" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="F10" t="s">
+      <c r="F10" s="1" t="s">
         <v>7</v>
       </c>
       <c r="G10" s="1" t="s">
@@ -657,16 +675,16 @@
       </c>
     </row>
     <row r="11" spans="2:7" x14ac:dyDescent="0.25">
-      <c r="B11" t="s">
+      <c r="B11" s="2" t="s">
         <v>8</v>
       </c>
       <c r="D11" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="E11" s="1" t="s">
+      <c r="E11" s="3" t="s">
         <v>8</v>
       </c>
-      <c r="F11" t="s">
+      <c r="F11" s="1" t="s">
         <v>8</v>
       </c>
       <c r="G11" s="1" t="s">
@@ -674,7 +692,7 @@
       </c>
     </row>
     <row r="12" spans="2:7" x14ac:dyDescent="0.25">
-      <c r="B12" t="s">
+      <c r="B12" s="2" t="s">
         <v>9</v>
       </c>
       <c r="D12" s="1" t="s">
@@ -683,7 +701,7 @@
       <c r="E12" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="F12" t="s">
+      <c r="F12" s="1" t="s">
         <v>9</v>
       </c>
       <c r="G12" s="1" t="s">
@@ -691,7 +709,7 @@
       </c>
     </row>
     <row r="13" spans="2:7" x14ac:dyDescent="0.25">
-      <c r="B13" t="s">
+      <c r="B13" s="2" t="s">
         <v>13</v>
       </c>
       <c r="D13" s="1" t="s">
@@ -700,7 +718,7 @@
       <c r="E13" s="1" t="s">
         <v>13</v>
       </c>
-      <c r="F13" t="s">
+      <c r="F13" s="1" t="s">
         <v>13</v>
       </c>
       <c r="G13" s="1" t="s">
@@ -708,7 +726,7 @@
       </c>
     </row>
     <row r="14" spans="2:7" x14ac:dyDescent="0.25">
-      <c r="B14" t="s">
+      <c r="B14" s="2" t="s">
         <v>14</v>
       </c>
       <c r="D14" s="1" t="s">
@@ -717,7 +735,7 @@
       <c r="E14" s="1" t="s">
         <v>14</v>
       </c>
-      <c r="F14" t="s">
+      <c r="F14" s="1" t="s">
         <v>14</v>
       </c>
       <c r="G14" s="1" t="s">
@@ -725,7 +743,7 @@
       </c>
     </row>
     <row r="15" spans="2:7" x14ac:dyDescent="0.25">
-      <c r="B15" t="s">
+      <c r="B15" s="2" t="s">
         <v>15</v>
       </c>
       <c r="D15" s="1" t="s">
@@ -734,7 +752,7 @@
       <c r="E15" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="F15" t="s">
+      <c r="F15" s="1" t="s">
         <v>15</v>
       </c>
       <c r="G15" s="1" t="s">
@@ -742,7 +760,7 @@
       </c>
     </row>
     <row r="16" spans="2:7" x14ac:dyDescent="0.25">
-      <c r="B16" t="s">
+      <c r="B16" s="2" t="s">
         <v>11</v>
       </c>
       <c r="D16" s="1" t="s">
@@ -751,7 +769,7 @@
       <c r="E16" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="F16" t="s">
+      <c r="F16" s="1" t="s">
         <v>11</v>
       </c>
       <c r="G16" s="1" t="s">
@@ -759,7 +777,7 @@
       </c>
     </row>
     <row r="17" spans="2:7" x14ac:dyDescent="0.25">
-      <c r="B17" t="s">
+      <c r="B17" s="2" t="s">
         <v>12</v>
       </c>
       <c r="D17" s="1" t="s">
@@ -768,7 +786,7 @@
       <c r="E17" s="1" t="s">
         <v>12</v>
       </c>
-      <c r="F17" t="s">
+      <c r="F17" s="1" t="s">
         <v>12</v>
       </c>
       <c r="G17" s="1" t="s">

</xml_diff>

<commit_message>
Finished all methods aside from new ones and wet chem
</commit_message>
<xml_diff>
--- a/Alike Columns.xlsx
+++ b/Alike Columns.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\kaleb\Desktop\LIMS\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{11B78F9B-F6AB-47E9-8D63-0D7AF3E01E7E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5FEC506F-E807-4F87-856E-E356DC4FB301}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-315" yWindow="-16320" windowWidth="29040" windowHeight="16440" xr2:uid="{360149B4-E1F2-4E19-BB44-4713DD98EAB8}"/>
+    <workbookView xWindow="28485" yWindow="-16410" windowWidth="29040" windowHeight="16440" xr2:uid="{360149B4-E1F2-4E19-BB44-4713DD98EAB8}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -157,11 +157,10 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="1"/>
     <xf numFmtId="0" fontId="2" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="0" xfId="1" applyFont="1" applyFill="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Good" xfId="1" builtinId="26"/>
@@ -681,7 +680,7 @@
       <c r="D11" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="E11" s="3" t="s">
+      <c r="E11" s="1" t="s">
         <v>8</v>
       </c>
       <c r="F11" s="1" t="s">

</xml_diff>